<commit_message>
feat: modernize import template and drop unused Player.email
Import template (MahjongTemplate.xlsx):
- unhide the Team, Random position and previously collapsed rows/columns
  (zeroHeight + hidden ranges) so the whole Players/Options grid is editable
- add the optional "Is round" column to the Schedule sheet, filled to match
  the example rounds

Import parser:
- read seating sheets formula-aware (data_only=False) and evaluate the mirror
  formulas ("=14+8"), rejecting a sheet that doesn't seat every competitor
  1..N exactly once per round instead of loading a half-empty chart
- treat the "Is round" column as optional, falling back to name-guessing

Remove Player.email everywhere: model field (+ migration 0011), import/export
columns, the player-editor column, and tests. It was collected but never used
to contact anyone and was leaking into stats output; dropping it is cleaner for
the public release. Golden snapshots regenerated (email-only removals).
</commit_message>
<xml_diff>
--- a/mahj/static/MahjongTemplate.xlsx
+++ b/mahj/static/MahjongTemplate.xlsx
@@ -472,7 +472,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B6"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="0"/>
   <cols>
     <col width="29.7109375" customWidth="1" style="1" min="1" max="1"/>
     <col width="87.85546875" customWidth="1" style="3" min="2" max="2"/>
@@ -17312,13 +17312,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="1"/>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15" zeroHeight="0"/>
   <cols>
     <col width="27.7109375" customWidth="1" style="3" min="1" max="3"/>
     <col width="40.42578125" customWidth="1" style="3" min="4" max="4"/>
-    <col hidden="1" width="40.42578125" customWidth="1" style="3" min="5" max="5"/>
-    <col hidden="1" width="40.42578125" customWidth="1" style="3" min="6" max="16384"/>
+    <col width="40.42578125" customWidth="1" min="5" max="5"/>
+    <col width="40.42578125" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="2">
@@ -17353,659 +17353,6 @@
         </is>
       </c>
     </row>
-    <row r="73" hidden="1"/>
-    <row r="74" hidden="1"/>
-    <row r="75" hidden="1"/>
-    <row r="76" hidden="1"/>
-    <row r="77" hidden="1"/>
-    <row r="78" hidden="1"/>
-    <row r="79" hidden="1"/>
-    <row r="80" hidden="1"/>
-    <row r="81" hidden="1"/>
-    <row r="82" hidden="1"/>
-    <row r="83" hidden="1"/>
-    <row r="84" hidden="1"/>
-    <row r="85" hidden="1"/>
-    <row r="86" hidden="1"/>
-    <row r="87" hidden="1"/>
-    <row r="88" hidden="1"/>
-    <row r="89" hidden="1"/>
-    <row r="90" hidden="1"/>
-    <row r="91" hidden="1"/>
-    <row r="92" hidden="1"/>
-    <row r="93" hidden="1"/>
-    <row r="94" hidden="1"/>
-    <row r="95" hidden="1"/>
-    <row r="96" hidden="1"/>
-    <row r="97" hidden="1"/>
-    <row r="98" hidden="1"/>
-    <row r="99" hidden="1"/>
-    <row r="100" hidden="1"/>
-    <row r="101" hidden="1"/>
-    <row r="102" hidden="1"/>
-    <row r="103" hidden="1"/>
-    <row r="104" hidden="1"/>
-    <row r="105" hidden="1"/>
-    <row r="106" hidden="1"/>
-    <row r="107" hidden="1"/>
-    <row r="108" hidden="1"/>
-    <row r="109" hidden="1"/>
-    <row r="110" hidden="1"/>
-    <row r="111" hidden="1"/>
-    <row r="112" hidden="1"/>
-    <row r="113" hidden="1"/>
-    <row r="114" hidden="1"/>
-    <row r="115" hidden="1"/>
-    <row r="116" hidden="1"/>
-    <row r="117" hidden="1"/>
-    <row r="118" hidden="1"/>
-    <row r="119" hidden="1"/>
-    <row r="120" hidden="1"/>
-    <row r="121" hidden="1"/>
-    <row r="122" hidden="1"/>
-    <row r="123" hidden="1"/>
-    <row r="124" hidden="1"/>
-    <row r="125" hidden="1"/>
-    <row r="126" hidden="1"/>
-    <row r="127" hidden="1"/>
-    <row r="128" hidden="1"/>
-    <row r="129" hidden="1"/>
-    <row r="130" hidden="1"/>
-    <row r="131" hidden="1"/>
-    <row r="132" hidden="1"/>
-    <row r="133" hidden="1"/>
-    <row r="134" hidden="1"/>
-    <row r="135" hidden="1"/>
-    <row r="136" hidden="1"/>
-    <row r="137" hidden="1"/>
-    <row r="138" hidden="1"/>
-    <row r="139" hidden="1"/>
-    <row r="140" hidden="1"/>
-    <row r="141" hidden="1"/>
-    <row r="142" hidden="1"/>
-    <row r="143" hidden="1"/>
-    <row r="144" hidden="1"/>
-    <row r="145" hidden="1"/>
-    <row r="146" hidden="1"/>
-    <row r="147" hidden="1"/>
-    <row r="148" hidden="1"/>
-    <row r="149" hidden="1"/>
-    <row r="150" hidden="1"/>
-    <row r="151" hidden="1"/>
-    <row r="152" hidden="1"/>
-    <row r="153" hidden="1"/>
-    <row r="154" hidden="1"/>
-    <row r="155" hidden="1"/>
-    <row r="156" hidden="1"/>
-    <row r="157" hidden="1"/>
-    <row r="158" hidden="1"/>
-    <row r="159" hidden="1"/>
-    <row r="160" hidden="1"/>
-    <row r="161" hidden="1"/>
-    <row r="162" hidden="1"/>
-    <row r="163" hidden="1"/>
-    <row r="164" hidden="1"/>
-    <row r="165" hidden="1"/>
-    <row r="166" hidden="1"/>
-    <row r="167" hidden="1"/>
-    <row r="168" hidden="1"/>
-    <row r="169" hidden="1"/>
-    <row r="170" hidden="1"/>
-    <row r="171" hidden="1"/>
-    <row r="172" hidden="1"/>
-    <row r="173" hidden="1"/>
-    <row r="174" hidden="1"/>
-    <row r="175" hidden="1"/>
-    <row r="176" hidden="1"/>
-    <row r="177" hidden="1"/>
-    <row r="178" hidden="1"/>
-    <row r="179" hidden="1"/>
-    <row r="180" hidden="1"/>
-    <row r="181" hidden="1"/>
-    <row r="182" hidden="1"/>
-    <row r="183" hidden="1"/>
-    <row r="184" hidden="1"/>
-    <row r="185" hidden="1"/>
-    <row r="186" hidden="1"/>
-    <row r="187" hidden="1"/>
-    <row r="188" hidden="1"/>
-    <row r="189" hidden="1"/>
-    <row r="190" hidden="1"/>
-    <row r="191" hidden="1"/>
-    <row r="192" hidden="1"/>
-    <row r="193" hidden="1"/>
-    <row r="194" hidden="1"/>
-    <row r="195" hidden="1"/>
-    <row r="196" hidden="1"/>
-    <row r="197" hidden="1"/>
-    <row r="198" hidden="1"/>
-    <row r="199" hidden="1"/>
-    <row r="200" hidden="1"/>
-    <row r="201" hidden="1"/>
-    <row r="202" hidden="1"/>
-    <row r="203" hidden="1"/>
-    <row r="204" hidden="1"/>
-    <row r="205" hidden="1"/>
-    <row r="206" hidden="1"/>
-    <row r="207" hidden="1"/>
-    <row r="208" hidden="1"/>
-    <row r="209" hidden="1"/>
-    <row r="210" hidden="1"/>
-    <row r="211" hidden="1"/>
-    <row r="212" hidden="1"/>
-    <row r="213" hidden="1"/>
-    <row r="214" hidden="1"/>
-    <row r="215" hidden="1"/>
-    <row r="216" hidden="1"/>
-    <row r="217" hidden="1"/>
-    <row r="218" hidden="1"/>
-    <row r="219" hidden="1"/>
-    <row r="220" hidden="1"/>
-    <row r="221" hidden="1"/>
-    <row r="222" hidden="1"/>
-    <row r="223" hidden="1"/>
-    <row r="224" hidden="1"/>
-    <row r="225" hidden="1"/>
-    <row r="226" hidden="1"/>
-    <row r="227" hidden="1"/>
-    <row r="228" hidden="1"/>
-    <row r="229" hidden="1"/>
-    <row r="230" hidden="1"/>
-    <row r="231" hidden="1"/>
-    <row r="232" hidden="1"/>
-    <row r="233" hidden="1"/>
-    <row r="234" hidden="1"/>
-    <row r="235" hidden="1"/>
-    <row r="236" hidden="1"/>
-    <row r="237" hidden="1"/>
-    <row r="238" hidden="1"/>
-    <row r="239" hidden="1"/>
-    <row r="240" hidden="1"/>
-    <row r="241" hidden="1"/>
-    <row r="242" hidden="1"/>
-    <row r="243" hidden="1"/>
-    <row r="244" hidden="1"/>
-    <row r="245" hidden="1"/>
-    <row r="246" hidden="1"/>
-    <row r="247" hidden="1"/>
-    <row r="248" hidden="1"/>
-    <row r="249" hidden="1"/>
-    <row r="250" hidden="1"/>
-    <row r="251" hidden="1"/>
-    <row r="252" hidden="1"/>
-    <row r="253" hidden="1"/>
-    <row r="254" hidden="1"/>
-    <row r="255" hidden="1"/>
-    <row r="256" hidden="1"/>
-    <row r="257" hidden="1"/>
-    <row r="258" hidden="1"/>
-    <row r="259" hidden="1"/>
-    <row r="260" hidden="1"/>
-    <row r="261" hidden="1"/>
-    <row r="262" hidden="1"/>
-    <row r="263" hidden="1"/>
-    <row r="264" hidden="1"/>
-    <row r="265" hidden="1"/>
-    <row r="266" hidden="1"/>
-    <row r="267" hidden="1"/>
-    <row r="268" hidden="1"/>
-    <row r="269" hidden="1"/>
-    <row r="270" hidden="1"/>
-    <row r="271" hidden="1"/>
-    <row r="272" hidden="1"/>
-    <row r="273" hidden="1"/>
-    <row r="274" hidden="1"/>
-    <row r="275" hidden="1"/>
-    <row r="276" hidden="1"/>
-    <row r="277" hidden="1"/>
-    <row r="278" hidden="1"/>
-    <row r="279" hidden="1"/>
-    <row r="280" hidden="1"/>
-    <row r="281" hidden="1"/>
-    <row r="282" hidden="1"/>
-    <row r="283" hidden="1"/>
-    <row r="284" hidden="1"/>
-    <row r="285" hidden="1"/>
-    <row r="286" hidden="1"/>
-    <row r="287" hidden="1"/>
-    <row r="288" hidden="1"/>
-    <row r="289" hidden="1"/>
-    <row r="290" hidden="1"/>
-    <row r="291" hidden="1"/>
-    <row r="292" hidden="1"/>
-    <row r="293" hidden="1"/>
-    <row r="294" hidden="1"/>
-    <row r="295" hidden="1"/>
-    <row r="296" hidden="1"/>
-    <row r="297" hidden="1"/>
-    <row r="298" hidden="1"/>
-    <row r="299" hidden="1"/>
-    <row r="300" hidden="1"/>
-    <row r="301" hidden="1"/>
-    <row r="302" hidden="1"/>
-    <row r="303" hidden="1"/>
-    <row r="304" hidden="1"/>
-    <row r="305" hidden="1"/>
-    <row r="306" hidden="1"/>
-    <row r="307" hidden="1"/>
-    <row r="308" hidden="1"/>
-    <row r="309" hidden="1"/>
-    <row r="310" hidden="1"/>
-    <row r="311" hidden="1"/>
-    <row r="312" hidden="1"/>
-    <row r="313" hidden="1"/>
-    <row r="314" hidden="1"/>
-    <row r="315" hidden="1"/>
-    <row r="316" hidden="1"/>
-    <row r="317" hidden="1"/>
-    <row r="318" hidden="1"/>
-    <row r="319" hidden="1"/>
-    <row r="320" hidden="1"/>
-    <row r="321" hidden="1"/>
-    <row r="322" hidden="1"/>
-    <row r="323" hidden="1"/>
-    <row r="324" hidden="1"/>
-    <row r="325" hidden="1"/>
-    <row r="326" hidden="1"/>
-    <row r="327" hidden="1"/>
-    <row r="328" hidden="1"/>
-    <row r="329" hidden="1"/>
-    <row r="330" hidden="1"/>
-    <row r="331" hidden="1"/>
-    <row r="332" hidden="1"/>
-    <row r="333" hidden="1"/>
-    <row r="334" hidden="1"/>
-    <row r="335" hidden="1"/>
-    <row r="336" hidden="1"/>
-    <row r="337" hidden="1"/>
-    <row r="338" hidden="1"/>
-    <row r="339" hidden="1"/>
-    <row r="340" hidden="1"/>
-    <row r="341" hidden="1"/>
-    <row r="342" hidden="1"/>
-    <row r="343" hidden="1"/>
-    <row r="344" hidden="1"/>
-    <row r="345" hidden="1"/>
-    <row r="346" hidden="1"/>
-    <row r="347" hidden="1"/>
-    <row r="348" hidden="1"/>
-    <row r="349" hidden="1"/>
-    <row r="350" hidden="1"/>
-    <row r="351" hidden="1"/>
-    <row r="352" hidden="1"/>
-    <row r="353" hidden="1"/>
-    <row r="354" hidden="1"/>
-    <row r="355" hidden="1"/>
-    <row r="356" hidden="1"/>
-    <row r="357" hidden="1"/>
-    <row r="358" hidden="1"/>
-    <row r="359" hidden="1"/>
-    <row r="360" hidden="1"/>
-    <row r="361" hidden="1"/>
-    <row r="362" hidden="1"/>
-    <row r="363" hidden="1"/>
-    <row r="364" hidden="1"/>
-    <row r="365" hidden="1"/>
-    <row r="366" hidden="1"/>
-    <row r="367" hidden="1"/>
-    <row r="368" hidden="1"/>
-    <row r="369" hidden="1"/>
-    <row r="370" hidden="1"/>
-    <row r="371" hidden="1"/>
-    <row r="372" hidden="1"/>
-    <row r="373" hidden="1"/>
-    <row r="374" hidden="1"/>
-    <row r="375" hidden="1"/>
-    <row r="376" hidden="1"/>
-    <row r="377" hidden="1"/>
-    <row r="378" hidden="1"/>
-    <row r="379" hidden="1"/>
-    <row r="380" hidden="1"/>
-    <row r="381" hidden="1"/>
-    <row r="382" hidden="1"/>
-    <row r="383" hidden="1"/>
-    <row r="384" hidden="1"/>
-    <row r="385" hidden="1"/>
-    <row r="386" hidden="1"/>
-    <row r="387" hidden="1"/>
-    <row r="388" hidden="1"/>
-    <row r="389" hidden="1"/>
-    <row r="390" hidden="1"/>
-    <row r="391" hidden="1"/>
-    <row r="392" hidden="1"/>
-    <row r="393" hidden="1"/>
-    <row r="394" hidden="1"/>
-    <row r="395" hidden="1"/>
-    <row r="396" hidden="1"/>
-    <row r="397" hidden="1"/>
-    <row r="398" hidden="1"/>
-    <row r="399" hidden="1"/>
-    <row r="400" hidden="1"/>
-    <row r="401" hidden="1"/>
-    <row r="402" hidden="1"/>
-    <row r="403" hidden="1"/>
-    <row r="404" hidden="1"/>
-    <row r="405" hidden="1"/>
-    <row r="406" hidden="1"/>
-    <row r="407" hidden="1"/>
-    <row r="408" hidden="1"/>
-    <row r="409" hidden="1"/>
-    <row r="410" hidden="1"/>
-    <row r="411" hidden="1"/>
-    <row r="412" hidden="1"/>
-    <row r="413" hidden="1"/>
-    <row r="414" hidden="1"/>
-    <row r="415" hidden="1"/>
-    <row r="416" hidden="1"/>
-    <row r="417" hidden="1"/>
-    <row r="418" hidden="1"/>
-    <row r="419" hidden="1"/>
-    <row r="420" hidden="1"/>
-    <row r="421" hidden="1"/>
-    <row r="422" hidden="1"/>
-    <row r="423" hidden="1"/>
-    <row r="424" hidden="1"/>
-    <row r="425" hidden="1"/>
-    <row r="426" hidden="1"/>
-    <row r="427" hidden="1"/>
-    <row r="428" hidden="1"/>
-    <row r="429" hidden="1"/>
-    <row r="430" hidden="1"/>
-    <row r="431" hidden="1"/>
-    <row r="432" hidden="1"/>
-    <row r="433" hidden="1"/>
-    <row r="434" hidden="1"/>
-    <row r="435" hidden="1"/>
-    <row r="436" hidden="1"/>
-    <row r="437" hidden="1"/>
-    <row r="438" hidden="1"/>
-    <row r="439" hidden="1"/>
-    <row r="440" hidden="1"/>
-    <row r="441" hidden="1"/>
-    <row r="442" hidden="1"/>
-    <row r="443" hidden="1"/>
-    <row r="444" hidden="1"/>
-    <row r="445" hidden="1"/>
-    <row r="446" hidden="1"/>
-    <row r="447" hidden="1"/>
-    <row r="448" hidden="1"/>
-    <row r="449" hidden="1"/>
-    <row r="450" hidden="1"/>
-    <row r="451" hidden="1"/>
-    <row r="452" hidden="1"/>
-    <row r="453" hidden="1"/>
-    <row r="454" hidden="1"/>
-    <row r="455" hidden="1"/>
-    <row r="456" hidden="1"/>
-    <row r="457" hidden="1"/>
-    <row r="458" hidden="1"/>
-    <row r="459" hidden="1"/>
-    <row r="460" hidden="1"/>
-    <row r="461" hidden="1"/>
-    <row r="462" hidden="1"/>
-    <row r="463" hidden="1"/>
-    <row r="464" hidden="1"/>
-    <row r="465" hidden="1"/>
-    <row r="466" hidden="1"/>
-    <row r="467" hidden="1"/>
-    <row r="468" hidden="1"/>
-    <row r="469" hidden="1"/>
-    <row r="470" hidden="1"/>
-    <row r="471" hidden="1"/>
-    <row r="472" hidden="1"/>
-    <row r="473" hidden="1"/>
-    <row r="474" hidden="1"/>
-    <row r="475" hidden="1"/>
-    <row r="476" hidden="1"/>
-    <row r="477" hidden="1"/>
-    <row r="478" hidden="1"/>
-    <row r="479" hidden="1"/>
-    <row r="480" hidden="1"/>
-    <row r="481" hidden="1"/>
-    <row r="482" hidden="1"/>
-    <row r="483" hidden="1"/>
-    <row r="484" hidden="1"/>
-    <row r="485" hidden="1"/>
-    <row r="486" hidden="1"/>
-    <row r="487" hidden="1"/>
-    <row r="488" hidden="1"/>
-    <row r="489" hidden="1"/>
-    <row r="490" hidden="1"/>
-    <row r="491" hidden="1"/>
-    <row r="492" hidden="1"/>
-    <row r="493" hidden="1"/>
-    <row r="494" hidden="1"/>
-    <row r="495" hidden="1"/>
-    <row r="496" hidden="1"/>
-    <row r="497" hidden="1"/>
-    <row r="498" hidden="1"/>
-    <row r="499" hidden="1"/>
-    <row r="500" hidden="1"/>
-    <row r="501" hidden="1"/>
-    <row r="502" hidden="1"/>
-    <row r="503" hidden="1"/>
-    <row r="504" hidden="1"/>
-    <row r="505" hidden="1"/>
-    <row r="506" hidden="1"/>
-    <row r="507" hidden="1"/>
-    <row r="508" hidden="1"/>
-    <row r="509" hidden="1"/>
-    <row r="510" hidden="1"/>
-    <row r="511" hidden="1"/>
-    <row r="512" hidden="1"/>
-    <row r="513" hidden="1"/>
-    <row r="514" hidden="1"/>
-    <row r="515" hidden="1"/>
-    <row r="516" hidden="1"/>
-    <row r="517" hidden="1"/>
-    <row r="518" hidden="1"/>
-    <row r="519" hidden="1"/>
-    <row r="520" hidden="1"/>
-    <row r="521" hidden="1"/>
-    <row r="522" hidden="1"/>
-    <row r="523" hidden="1"/>
-    <row r="524" hidden="1"/>
-    <row r="525" hidden="1"/>
-    <row r="526" hidden="1"/>
-    <row r="527" hidden="1"/>
-    <row r="528" hidden="1"/>
-    <row r="529" hidden="1"/>
-    <row r="530" hidden="1"/>
-    <row r="531" hidden="1"/>
-    <row r="532" hidden="1"/>
-    <row r="533" hidden="1"/>
-    <row r="534" hidden="1"/>
-    <row r="535" hidden="1"/>
-    <row r="536" hidden="1"/>
-    <row r="537" hidden="1"/>
-    <row r="538" hidden="1"/>
-    <row r="539" hidden="1"/>
-    <row r="540" hidden="1"/>
-    <row r="541" hidden="1"/>
-    <row r="542" hidden="1"/>
-    <row r="543" hidden="1"/>
-    <row r="544" hidden="1"/>
-    <row r="545" hidden="1"/>
-    <row r="546" hidden="1"/>
-    <row r="547" hidden="1"/>
-    <row r="548" hidden="1"/>
-    <row r="549" hidden="1"/>
-    <row r="550" hidden="1"/>
-    <row r="551" hidden="1"/>
-    <row r="552" hidden="1"/>
-    <row r="553" hidden="1"/>
-    <row r="554" hidden="1"/>
-    <row r="555" hidden="1"/>
-    <row r="556" hidden="1"/>
-    <row r="557" hidden="1"/>
-    <row r="558" hidden="1"/>
-    <row r="559" hidden="1"/>
-    <row r="560" hidden="1"/>
-    <row r="561" hidden="1"/>
-    <row r="562" hidden="1"/>
-    <row r="563" hidden="1"/>
-    <row r="564" hidden="1"/>
-    <row r="565" hidden="1"/>
-    <row r="566" hidden="1"/>
-    <row r="567" hidden="1"/>
-    <row r="568" hidden="1"/>
-    <row r="569" hidden="1"/>
-    <row r="570" hidden="1"/>
-    <row r="571" hidden="1"/>
-    <row r="572" hidden="1"/>
-    <row r="573" hidden="1"/>
-    <row r="574" hidden="1"/>
-    <row r="575" hidden="1"/>
-    <row r="576" hidden="1"/>
-    <row r="577" hidden="1"/>
-    <row r="578" hidden="1"/>
-    <row r="579" hidden="1"/>
-    <row r="580" hidden="1"/>
-    <row r="581" hidden="1"/>
-    <row r="582" hidden="1"/>
-    <row r="583" hidden="1"/>
-    <row r="584" hidden="1"/>
-    <row r="585" hidden="1"/>
-    <row r="586" hidden="1"/>
-    <row r="587" hidden="1"/>
-    <row r="588" hidden="1"/>
-    <row r="589" hidden="1"/>
-    <row r="590" hidden="1"/>
-    <row r="591" hidden="1"/>
-    <row r="592" hidden="1"/>
-    <row r="593" hidden="1"/>
-    <row r="594" hidden="1"/>
-    <row r="595" hidden="1"/>
-    <row r="596" hidden="1"/>
-    <row r="597" hidden="1"/>
-    <row r="598" hidden="1"/>
-    <row r="599" hidden="1"/>
-    <row r="600" hidden="1"/>
-    <row r="601" hidden="1"/>
-    <row r="602" hidden="1"/>
-    <row r="603" hidden="1"/>
-    <row r="604" hidden="1"/>
-    <row r="605" hidden="1"/>
-    <row r="606" hidden="1"/>
-    <row r="607" hidden="1"/>
-    <row r="608" hidden="1"/>
-    <row r="609" hidden="1"/>
-    <row r="610" hidden="1"/>
-    <row r="611" hidden="1"/>
-    <row r="612" hidden="1"/>
-    <row r="613" hidden="1"/>
-    <row r="614" hidden="1"/>
-    <row r="615" hidden="1"/>
-    <row r="616" hidden="1"/>
-    <row r="617" hidden="1"/>
-    <row r="618" hidden="1"/>
-    <row r="619" hidden="1"/>
-    <row r="620" hidden="1"/>
-    <row r="621" hidden="1"/>
-    <row r="622" hidden="1"/>
-    <row r="623" hidden="1"/>
-    <row r="624" hidden="1"/>
-    <row r="625" hidden="1"/>
-    <row r="626" hidden="1"/>
-    <row r="627" hidden="1"/>
-    <row r="628" hidden="1"/>
-    <row r="629" hidden="1"/>
-    <row r="630" hidden="1"/>
-    <row r="631" hidden="1"/>
-    <row r="632" hidden="1"/>
-    <row r="633" hidden="1"/>
-    <row r="634" hidden="1"/>
-    <row r="635" hidden="1"/>
-    <row r="636" hidden="1"/>
-    <row r="637" hidden="1"/>
-    <row r="638" hidden="1"/>
-    <row r="639" hidden="1"/>
-    <row r="640" hidden="1"/>
-    <row r="641" hidden="1"/>
-    <row r="642" hidden="1"/>
-    <row r="643" hidden="1"/>
-    <row r="644" hidden="1"/>
-    <row r="645" hidden="1"/>
-    <row r="646" hidden="1"/>
-    <row r="647" hidden="1"/>
-    <row r="648" hidden="1"/>
-    <row r="649" hidden="1"/>
-    <row r="650" hidden="1"/>
-    <row r="651" hidden="1"/>
-    <row r="652" hidden="1"/>
-    <row r="653" hidden="1"/>
-    <row r="654" hidden="1"/>
-    <row r="655" hidden="1"/>
-    <row r="656" hidden="1"/>
-    <row r="657" hidden="1"/>
-    <row r="658" hidden="1"/>
-    <row r="659" hidden="1"/>
-    <row r="660" hidden="1"/>
-    <row r="661" hidden="1"/>
-    <row r="662" hidden="1"/>
-    <row r="663" hidden="1"/>
-    <row r="664" hidden="1"/>
-    <row r="665" hidden="1"/>
-    <row r="666" hidden="1"/>
-    <row r="667" hidden="1"/>
-    <row r="668" hidden="1"/>
-    <row r="669" hidden="1"/>
-    <row r="670" hidden="1"/>
-    <row r="671" hidden="1"/>
-    <row r="672" hidden="1"/>
-    <row r="673" hidden="1"/>
-    <row r="674" hidden="1"/>
-    <row r="675" hidden="1"/>
-    <row r="676" hidden="1"/>
-    <row r="677" hidden="1"/>
-    <row r="678" hidden="1"/>
-    <row r="679" hidden="1"/>
-    <row r="680" hidden="1"/>
-    <row r="681" hidden="1"/>
-    <row r="682" hidden="1"/>
-    <row r="683" hidden="1"/>
-    <row r="684" hidden="1"/>
-    <row r="685" hidden="1"/>
-    <row r="686" hidden="1"/>
-    <row r="687" hidden="1"/>
-    <row r="688" hidden="1"/>
-    <row r="689" hidden="1"/>
-    <row r="690" hidden="1"/>
-    <row r="691" hidden="1"/>
-    <row r="692" hidden="1"/>
-    <row r="693" hidden="1"/>
-    <row r="694" hidden="1"/>
-    <row r="695" hidden="1"/>
-    <row r="696" hidden="1"/>
-    <row r="697" hidden="1"/>
-    <row r="698" hidden="1"/>
-    <row r="699" hidden="1"/>
-    <row r="700" hidden="1"/>
-    <row r="701" hidden="1"/>
-    <row r="702" hidden="1"/>
-    <row r="703" hidden="1"/>
-    <row r="704" hidden="1"/>
-    <row r="705" hidden="1"/>
-    <row r="706" hidden="1"/>
-    <row r="707" hidden="1"/>
-    <row r="708" hidden="1"/>
-    <row r="709" hidden="1"/>
-    <row r="710" hidden="1"/>
-    <row r="711" hidden="1"/>
-    <row r="712" hidden="1"/>
-    <row r="713" hidden="1"/>
-    <row r="714" hidden="1"/>
-    <row r="715" hidden="1"/>
-    <row r="716" hidden="1"/>
-    <row r="717" hidden="1"/>
-    <row r="718" hidden="1"/>
-    <row r="719" hidden="1"/>
-    <row r="720" hidden="1"/>
-    <row r="721" hidden="1"/>
-    <row r="722" hidden="1"/>
-    <row r="723" hidden="1"/>
-    <row r="724" hidden="1"/>
-    <row r="725" hidden="1"/>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:XFD72" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" type="custom">
@@ -18023,13 +17370,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="0" defaultRowHeight="15"/>
   <cols>
     <col width="21.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="16.42578125" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
-    <col hidden="1" width="9.140625" customWidth="1" min="4" max="16384"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="1" s="1">
@@ -18048,6 +17395,11 @@
           <t>Name</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Is round</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -18065,6 +17417,9 @@
           <t>Registration and info</t>
         </is>
       </c>
+      <c r="D2" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -18082,6 +17437,9 @@
           <t>Round 1</t>
         </is>
       </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -18099,6 +17457,9 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="D4" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -18116,6 +17477,9 @@
           <t>Round 2</t>
         </is>
       </c>
+      <c r="D5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -18133,6 +17497,9 @@
           <t>Lunch</t>
         </is>
       </c>
+      <c r="D6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -18150,6 +17517,9 @@
           <t>Round 3</t>
         </is>
       </c>
+      <c r="D7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -18167,6 +17537,9 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="D8" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -18184,6 +17557,9 @@
           <t>Round 4</t>
         </is>
       </c>
+      <c r="D9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -18201,6 +17577,9 @@
           <t>Registration day 2</t>
         </is>
       </c>
+      <c r="D10" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -18218,6 +17597,9 @@
           <t>Round 5</t>
         </is>
       </c>
+      <c r="D11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -18235,6 +17617,9 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="D12" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -18252,6 +17637,9 @@
           <t>Round 6</t>
         </is>
       </c>
+      <c r="D13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -18269,6 +17657,9 @@
           <t>Lunch</t>
         </is>
       </c>
+      <c r="D14" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -18286,6 +17677,9 @@
           <t>Round 7</t>
         </is>
       </c>
+      <c r="D15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -18303,6 +17697,9 @@
           <t>Coffee break</t>
         </is>
       </c>
+      <c r="D16" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -18319,6 +17716,9 @@
         <is>
           <t>Award Ceremony</t>
         </is>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>